<commit_message>
Refactor app structure and reorganize patterns
</commit_message>
<xml_diff>
--- a/timeinvariance.xlsx
+++ b/timeinvariance.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PilgrimBeart\git\neuron2025\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ABFE90-52C3-44A8-A1CD-E2463B6D11EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="22720" windowHeight="14480" xr2:uid="{16D0F2AB-7828-4F97-BC08-FFEECF2D0B17}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -80,8 +74,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,9 +127,9 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -147,6 +141,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -261,7 +256,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-6205-4521-A286-5A1BC6055F6F}"/>
             </c:ext>
@@ -346,7 +341,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-6205-4521-A286-5A1BC6055F6F}"/>
             </c:ext>
@@ -361,11 +356,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="726883231"/>
-        <c:axId val="726885631"/>
+        <c:axId val="635164752"/>
+        <c:axId val="635165296"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="726883231"/>
+        <c:axId val="635164752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -407,7 +402,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="726885631"/>
+        <c:crossAx val="635165296"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -415,7 +410,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="726885631"/>
+        <c:axId val="635165296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -466,7 +461,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="726883231"/>
+        <c:crossAx val="635164752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -480,6 +475,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -511,14 +507,14 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1129,7 +1125,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{208932B0-CE4F-06A7-D30D-22F8D1D921EE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{208932B0-CE4F-06A7-D30D-22F8D1D921EE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1466,41 +1462,41 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6758EA08-3173-48DF-9EAB-BD10309D8F80}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1514,12 +1510,12 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="D10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1533,7 +1529,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>0</v>
       </c>
@@ -1548,9 +1544,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6">
       <c r="A13">
-        <f>A12*(1-$C$9)+$B$12*($C$9)</f>
+        <f t="shared" ref="A13:A29" si="0">A12*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.1</v>
       </c>
       <c r="D13">
@@ -1558,236 +1554,237 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <f t="shared" ref="E13:E29" si="0">$B$12 + (0 - $B$12) * EXP(-$F$9*D13)</f>
+        <f t="shared" ref="E13:E29" si="1">$B$12 + (0 - $B$12) * EXP(-$F$9*D13)</f>
         <v>9.5162581964040482E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6">
       <c r="A14">
-        <f>A13*(1-$C$9)+$B$12*($C$9)</f>
+        <f t="shared" si="0"/>
         <v>0.19</v>
       </c>
       <c r="D14">
-        <f t="shared" ref="D14:D29" si="1">D13+1</f>
+        <f t="shared" ref="D14:D29" si="2">D13+1</f>
         <v>2</v>
       </c>
       <c r="E14">
+        <f t="shared" si="1"/>
+        <v>0.18126924692201818</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
         <f t="shared" si="0"/>
-        <v>0.18126924692201818</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <f>A14*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.27100000000000002</v>
       </c>
       <c r="D15">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="E15">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="E15">
+        <v>0.25918177931828212</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16">
         <f t="shared" si="0"/>
-        <v>0.25918177931828212</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <f>A15*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.34390000000000004</v>
       </c>
       <c r="D16">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="E16">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="E16">
+        <v>0.32967995396436067</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17">
         <f t="shared" si="0"/>
-        <v>0.32967995396436067</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <f>A16*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.40951000000000004</v>
       </c>
       <c r="D17">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="E17">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="E17">
+        <v>0.39346934028736658</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18">
         <f t="shared" si="0"/>
-        <v>0.39346934028736658</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <f>A17*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.46855900000000006</v>
       </c>
       <c r="D18">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="E18">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="E18">
+        <v>0.45118836390597361</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19">
         <f t="shared" si="0"/>
-        <v>0.45118836390597361</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <f>A18*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.52170310000000009</v>
       </c>
       <c r="D19">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="E19">
         <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-      <c r="E19">
+        <v>0.50341469620859058</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20">
         <f t="shared" si="0"/>
-        <v>0.50341469620859058</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <f>A19*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.56953279000000012</v>
       </c>
       <c r="D20">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="E20">
         <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="E20">
+        <v>0.55067103588277844</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21">
         <f t="shared" si="0"/>
-        <v>0.55067103588277844</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <f>A20*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.61257951100000008</v>
       </c>
       <c r="D21">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="E21">
         <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="E21">
+        <v>0.59343034025940089</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22">
         <f t="shared" si="0"/>
-        <v>0.59343034025940089</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <f>A21*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.65132155990000007</v>
       </c>
       <c r="D22">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="E22">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="E22">
+        <v>0.63212055882855767</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23">
         <f t="shared" si="0"/>
-        <v>0.63212055882855767</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <f>A22*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.68618940391000005</v>
       </c>
       <c r="D23">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="E23">
         <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-      <c r="E23">
+        <v>0.6671289163019205</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24">
         <f t="shared" si="0"/>
-        <v>0.6671289163019205</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <f>A23*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.717570463519</v>
       </c>
       <c r="D24">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="E24">
         <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="E24">
+        <v>0.69880578808779803</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25">
         <f t="shared" si="0"/>
-        <v>0.69880578808779803</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <f>A24*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.74581341716710003</v>
       </c>
       <c r="D25">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="E25">
         <f t="shared" si="1"/>
-        <v>13</v>
-      </c>
-      <c r="E25">
+        <v>0.72746820696598746</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26">
         <f t="shared" si="0"/>
-        <v>0.72746820696598746</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <f>A25*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.77123207545039008</v>
       </c>
       <c r="D26">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="E26">
         <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-      <c r="E26">
+        <v>0.75340303605839354</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27">
         <f t="shared" si="0"/>
-        <v>0.75340303605839354</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <f>A26*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.79410886790535107</v>
       </c>
       <c r="D27">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="E27">
         <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="E27">
+        <v>0.77686983985157021</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28">
         <f t="shared" si="0"/>
-        <v>0.77686983985157021</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <f>A27*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.81469798111481595</v>
       </c>
       <c r="D28">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="E28">
         <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="E28">
+        <v>0.79810348200534464</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29">
         <f t="shared" si="0"/>
-        <v>0.79810348200534464</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <f>A28*(1-$C$9)+$B$12*($C$9)</f>
         <v>0.83322818300333434</v>
       </c>
       <c r="D29">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+      <c r="E29">
         <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-      <c r="E29">
-        <f t="shared" si="0"/>
         <v>0.81731647594726542</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>